<commit_message>
Replace Disrupt with Flash Bang (Weaken 3) + balance-verify
Disrupt's text was a lie — the engine retimed the enemy's T4 attack to T3,
which resolves *earlier*, buffing the enemy. Replaced with Flash Bang:
T1 Spell, "Weaken 3 on one enemy." Reuses the suppress/turn.outgoing handler
(generalized to read `amount`); no new mechanic, class stays at 20 cards.

Balance (6,000 heuristic-mirror matches, A/B vs old Disrupt):
  Wraith 47.1% -> 48.7% (+1.6), tied-lowest -> mid-pack
  all other classes within -0.2..-0.5 (noise)
  band 46.6-50.2%, spread 3.6 pts -> no class out of line, no tuning needed

Regenerated the xlsx. Engine 12/12 + 20/20 green; browser-verified Flash Bang
in Wraith's deck ("Weaken 3 on one enemy."), 0 console errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Rift_Protocol_Card_Reference.xlsx
+++ b/Rift_Protocol_Card_Reference.xlsx
@@ -3324,7 +3324,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Disrupt</t>
+          <t>Flash Bang</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3345,14 +3345,17 @@
           <t>enemy</t>
         </is>
       </c>
+      <c r="G58" t="n">
+        <v>3</v>
+      </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>One enemy's T4 attack resolves at T3.</t>
+          <t>Weaken 3 on one enemy.</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Knock the timing off.</t>
+          <t>A white flash, and their aim is gone.</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8724,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Disrupt</t>
+          <t>Flash Bang</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -8742,14 +8745,17 @@
           <t>enemy</t>
         </is>
       </c>
+      <c r="G18" t="n">
+        <v>3</v>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>One enemy's T4 attack resolves at T3.</t>
+          <t>Weaken 3 on one enemy.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Knock the timing off.</t>
+          <t>A white flash, and their aim is gone.</t>
         </is>
       </c>
     </row>

</xml_diff>